<commit_message>
Temas mas consultados: agregar Q de mensajes al ranking del tablero
Pedido de la Direccion. El ranking salia solo con los nombres de las
categorias; ahora lleva el conteo exacto.

- calcular_conteo_categorias() devuelve ademas el conteo crudo del ultimo mes.
  Va aparte para no alterar 'resultado', que se escribe tal cual en la hoja
  'Comparativo' del reporte_mensajes. Ese Excel sale igual que antes.
- construir_ranking_texto() acepta el conteo como argumento OPCIONAL: sin el,
  devuelve el formato viejo. Por eso Temas_Consultados_Anual.py, que importa
  la funcion y la llama con un solo argumento, sigue funcionando.
- Encabezado 'Q de mensajes' (constante ENCABEZADO_UNIDAD_RANKING): en el
  tablero esta celda queda al lado de 'Contenidos mas consultados', que cuenta
  SESIONES. Son unidades distintas y no son comparables ni sumables.

Septiembre 2026 regenerado con numeros.
</commit_message>
<xml_diff>
--- a/Temas_Consultados/output/ranking_temas_consultados_septiembre_2026.xlsx
+++ b/Temas_Consultados/output/ranking_temas_consultados_septiembre_2026.xlsx
@@ -470,16 +470,17 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>1-Infracciones y Multas
-2-Trámites y Reclamos
-3-Salud (Médicos/Salud)
-4-Turnos (Generales)
-5-Movilidad + Estacionamiento
-6-Licencia de Conducir
-7-Impuestos (AGIP / Patentes / ABL)
-8-MIBA y Validación
-9-Educación (Inscripciones/Becas)
-10-Interacción Humana (Chatear)</t>
+          <t>Q de mensajes
+1-Infracciones y Multas: (169.362)
+2-Trámites y Reclamos: (122.697)
+3-Salud (Médicos/Salud): (109.106)
+4-Turnos (Generales): (99.706)
+5-Movilidad + Estacionamiento: (80.186)
+6-Licencia de Conducir: (64.435)
+7-Impuestos (AGIP / Patentes / ABL): (42.316)
+8-MIBA y Validación: (31.977)
+9-Educación (Inscripciones/Becas): (28.748)
+10-Interacción Humana (Chatear): (26.913)</t>
         </is>
       </c>
     </row>

</xml_diff>